<commit_message>
feat: add candidate numbers for round 2 voting
</commit_message>
<xml_diff>
--- a/2차_후보자_프로필_최종_정상수정_v6.xlsx
+++ b/2차_후보자_프로필_최종_정상수정_v6.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="171">
   <si>
     <t>사진</t>
   </si>
@@ -41,7 +41,8 @@
 청년2부 (21)</t>
   </si>
   <si>
-    <t/>
+    <t xml:space="preserve">배우자: 이유정
+가족: 기현승</t>
   </si>
   <si>
     <t>5교구</t>
@@ -54,6 +55,10 @@
 목장지기 (24~26)
 소년2부 (21)
 시온찬양대 (21~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 원현주
+가족: (기범진)(기영욱)</t>
   </si>
   <si>
     <t>2교구</t>
@@ -70,12 +75,19 @@
 희망나눔부 (21~26)</t>
   </si>
   <si>
+    <t>배우자: 이명희</t>
+  </si>
+  <si>
     <t>김영수</t>
   </si>
   <si>
     <t xml:space="preserve">관리부 (21~25)
 미화부 (21)
 희망나눔부 (21~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 김은미
+가족: (김설아)(김보인)(김보혜)</t>
   </si>
   <si>
     <t>이경진</t>
@@ -89,6 +101,10 @@
 희망나눔부 (22~23)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김미선B
+가족: (이예림)(이예성)</t>
+  </si>
+  <si>
     <t>정주영</t>
   </si>
   <si>
@@ -99,12 +115,19 @@
 해외선교부 (22~23)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김성일
+가족: 정우성</t>
+  </si>
+  <si>
     <t>최성욱</t>
   </si>
   <si>
     <t xml:space="preserve">목장지기 (22~24)
 차량봉사부 (21~26)
 희망나눔부 (21~23)</t>
+  </si>
+  <si>
+    <t>배우자: 전미영</t>
   </si>
   <si>
     <t>4교구</t>
@@ -121,6 +144,10 @@
 청년1부 (22~23)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 박종혜
+가족: (허성모)허람희, 허율희, 허민희, 허재희</t>
+  </si>
+  <si>
     <t>6교구</t>
   </si>
   <si>
@@ -129,6 +156,10 @@
   <si>
     <t xml:space="preserve">목장지기 (22~26)
 시온찬양대 (23~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 박세라
+가족: 권도원, 권유원</t>
   </si>
   <si>
     <t>권현달</t>
@@ -141,12 +172,20 @@
 희망나눔부 (23~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김선
+가족: 권성은, 권성훈</t>
+  </si>
+  <si>
     <t>김성운</t>
   </si>
   <si>
     <t xml:space="preserve">목장지기 (24~25)
 상례부 (23)
 통합미취학부 (23~24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 유순천
+가족: 김치원, 김승원</t>
   </si>
   <si>
     <t>김영문</t>
@@ -158,6 +197,10 @@
 청소년선교부 (24~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 정순정
+가족: 박운임, 김수안, 김수혁, 김수현E</t>
+  </si>
+  <si>
     <t>1교구</t>
   </si>
   <si>
@@ -165,6 +208,10 @@
   </si>
   <si>
     <t>글로리아찬양대 (21~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 이정미A
+가족: 김가음, 김하음, 김지음</t>
   </si>
   <si>
     <t>김용수</t>
@@ -172,6 +219,10 @@
   <si>
     <t xml:space="preserve">목장지기 (21~25)
 시온찬양대 (24~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 손은미
+가족: 김주희A, 김진A, 김지성</t>
   </si>
   <si>
     <t>김종원A</t>
@@ -182,12 +233,20 @@
 친교봉사부 (22)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김미라
+가족: 김동명, 김송다</t>
+  </si>
+  <si>
     <t>김효원</t>
   </si>
   <si>
     <t xml:space="preserve">3부예배부 (24)
 예배부 (25)
 차량봉사부 (21~23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 고미경
+가족: 김초연, 김삼건, 김건화</t>
   </si>
   <si>
     <t>류택건</t>
@@ -200,6 +259,10 @@
 희망나눔부 (22~23)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 최경희
+가족: (류진)(류현준)(류장건)</t>
+  </si>
+  <si>
     <t>박완석</t>
   </si>
   <si>
@@ -208,6 +271,10 @@
 차량봉사부 (24)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 정진은
+가족: (박재우)(박재형)</t>
+  </si>
+  <si>
     <t>박해준</t>
   </si>
   <si>
@@ -215,11 +282,19 @@
 유치부 (21~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 박소연
+가족: 박동현, (박서현)</t>
+  </si>
+  <si>
     <t>안상준</t>
   </si>
   <si>
     <t xml:space="preserve">시온찬양대 (21~26)
 청소년선교부 (24~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 신소연
+가족: 안정인</t>
   </si>
   <si>
     <t>양향우</t>
@@ -232,12 +307,20 @@
 희망나눔부 (23~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김경희C
+가족: 양희우</t>
+  </si>
+  <si>
     <t>유영선</t>
   </si>
   <si>
     <t xml:space="preserve">목장지기 (21~26)
 해외선교1부 (24~25)
 해외선교부 (23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 안보경
+가족: 유원정</t>
   </si>
   <si>
     <t>이동수</t>
@@ -249,12 +332,20 @@
 사랑나눔부 (22~23)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김인숙C
+가족: 이재훈, 이예빈</t>
+  </si>
+  <si>
     <t>이성현</t>
   </si>
   <si>
     <t xml:space="preserve">글로리아찬양대 (21~26)
 목장지기 (26)
 재정부 (22~23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 호혜정
+가족: (이결)이강B</t>
   </si>
   <si>
     <t>이주현B</t>
@@ -269,6 +360,9 @@
 희망나눔부 (24~26)</t>
   </si>
   <si>
+    <t>배우자: 김상숙</t>
+  </si>
+  <si>
     <t>전헌효</t>
   </si>
   <si>
@@ -279,6 +373,10 @@
 희망나눔부 (26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김명선
+가족: 전성민, 전민규</t>
+  </si>
+  <si>
     <t>3교구</t>
   </si>
   <si>
@@ -288,6 +386,10 @@
     <t xml:space="preserve">따뜻한한끼봉사부 (25)
 목장지기 (23~26)
 미화부 (21)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 박지현A
+가족: 정연우, 정연찬</t>
   </si>
   <si>
     <t>정우철</t>
@@ -299,6 +401,10 @@
 희망나눔부 (21~24)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 홍은혜A
+가족: 정다영, 정다원, 정세연</t>
+  </si>
+  <si>
     <t>주승열</t>
   </si>
   <si>
@@ -307,12 +413,19 @@
 학원선교부 (21)</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>최재필</t>
   </si>
   <si>
     <t xml:space="preserve">목장지기 (21~25)
 소년부 (24~26)
 의료선교부 (21~23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 박성은A
+가족: 최여안, 최온새미</t>
   </si>
   <si>
     <t>현상수</t>
@@ -324,11 +437,19 @@
 차량봉사부 (23~24)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김명원
+가족: 현소라, 현동훈</t>
+  </si>
+  <si>
     <t>고여진</t>
   </si>
   <si>
     <t xml:space="preserve">목장지기 (21~26)
 시온찬양대 (23~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 문현우
+가족: 문예은, 문예린</t>
   </si>
   <si>
     <t>권미득</t>
@@ -338,6 +459,10 @@
 영유아부 (21~26)
 청소년선교부 (23~26)
 학원선교부 (21)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 이성용
+가족: 이주원B, 이효원</t>
   </si>
   <si>
     <t>김경희A</t>
@@ -348,6 +473,10 @@
 유년1부 (21~22)
 중보기도부 (21~25)
 통합아동부 (23~25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 임경연
+가족: 임하윤, 임하란</t>
   </si>
   <si>
     <t>김명선</t>
@@ -360,6 +489,10 @@
 상례부 (22~23)
 시온찬양대 (24~26)
 중보기도부 (24~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 전헌효
+가족: 전성민, 전민규</t>
   </si>
   <si>
     <t>김상숙</t>
@@ -376,6 +509,9 @@
 중보기도부 (24~25)</t>
   </si>
   <si>
+    <t>배우자: 이주현B</t>
+  </si>
+  <si>
     <t>김선</t>
   </si>
   <si>
@@ -386,6 +522,10 @@
 희망나눔부 (25~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 권현달
+가족: 권성은, 권성훈</t>
+  </si>
+  <si>
     <t>김선옥</t>
   </si>
   <si>
@@ -394,6 +534,9 @@
 해외선교1부 (24~25)</t>
   </si>
   <si>
+    <t>가족: 이고은B</t>
+  </si>
+  <si>
     <t>김현경</t>
   </si>
   <si>
@@ -410,11 +553,19 @@
 중보기도부 (21~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 강상희
+가족: 강신승</t>
+  </si>
+  <si>
     <t>박규분</t>
   </si>
   <si>
     <t xml:space="preserve">따뜻한한끼봉사부 (25)
 목장지기 (22~25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: (도정택)
+가족: (도승욱)도소정</t>
   </si>
   <si>
     <t>박세정</t>
@@ -426,6 +577,10 @@
 통합아동부 (25~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 김형구
+가족: 김지유, 김온유B</t>
+  </si>
+  <si>
     <t>백금주</t>
   </si>
   <si>
@@ -435,6 +590,10 @@
 중보기도부 (21~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 이재광
+가족: 이정륜, 이용준</t>
+  </si>
+  <si>
     <t>사미자</t>
   </si>
   <si>
@@ -443,12 +602,19 @@
 중보기도부 (24~26)</t>
   </si>
   <si>
+    <t>배우자: 김용주</t>
+  </si>
+  <si>
     <t>손은미</t>
   </si>
   <si>
     <t xml:space="preserve">목장지기 (21~25)
 시온찬양대 (24~26)
 원더풀시니어부 (25~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 김용수
+가족: 김주희A, 김진A, 김지성</t>
   </si>
   <si>
     <t>안보경</t>
@@ -459,6 +625,10 @@
 학원선교부 (21)
 해외선교1부 (24~25)
 해외선교부 (23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 유영선
+가족: 유원정</t>
   </si>
   <si>
     <t>양혜선A</t>
@@ -476,6 +646,10 @@
 희망나눔부 (25)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 차종호
+가족: 차하빈</t>
+  </si>
+  <si>
     <t>윤혜영A</t>
   </si>
   <si>
@@ -487,12 +661,19 @@
 통합아동부 (23~24)</t>
   </si>
   <si>
+    <t>배우자: 신현석</t>
+  </si>
+  <si>
     <t>이성실A</t>
   </si>
   <si>
     <t xml:space="preserve">목장지기 (26)
 소년1부 (21~22)
 통합아동부 (23~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 한지환
+가족: 한필우</t>
   </si>
   <si>
     <t>임은희</t>
@@ -503,6 +684,9 @@
 시온찬양대 (22~26)
 씨앗학교 (21~22)
 청소년선교부 (23~25)</t>
+  </si>
+  <si>
+    <t>가족: 신난미, 신동혁</t>
   </si>
   <si>
     <t>전미영</t>
@@ -514,6 +698,9 @@
 시온찬양대 (21~26)
 차량봉사부 (24~26)
 청소년선교부 (26)</t>
+  </si>
+  <si>
+    <t>배우자: 최성욱</t>
   </si>
   <si>
     <t>차창복</t>
@@ -536,6 +723,10 @@
 중보기도부 (21~26)</t>
   </si>
   <si>
+    <t xml:space="preserve">배우자: 류택건
+가족: (류진)(류현준)(류장건)</t>
+  </si>
+  <si>
     <t>함은미</t>
   </si>
   <si>
@@ -544,6 +735,10 @@
 영유아1부 (22)
 중보기도부 (21~25)
 통합미취학부 (23~26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배우자: 백정일
+가족: 백재욱, 백민욱</t>
   </si>
 </sst>
 </file>
@@ -3099,21 +3294,21 @@
         <v>10</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>8</v>
@@ -3121,72 +3316,72 @@
     </row>
     <row r="5" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -3227,27 +3422,27 @@
     </row>
     <row r="2" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>8</v>
@@ -3255,209 +3450,209 @@
     </row>
     <row r="4" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>7</v>
+        <v>66</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>7</v>
+        <v>72</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>7</v>
+        <v>81</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>7</v>
+        <v>84</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>8</v>
@@ -3465,86 +3660,86 @@
     </row>
     <row r="19" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>7</v>
+        <v>91</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>7</v>
+        <v>94</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>7</v>
+        <v>100</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>7</v>
+        <v>103</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -3585,27 +3780,27 @@
     </row>
     <row r="2" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>106</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>76</v>
+        <v>107</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>7</v>
+        <v>109</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>8</v>
@@ -3613,41 +3808,41 @@
     </row>
     <row r="4" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>112</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>7</v>
+        <v>115</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>7</v>
+        <v>118</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>8</v>
@@ -3655,13 +3850,13 @@
     </row>
     <row r="7" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>8</v>
@@ -3669,83 +3864,83 @@
     </row>
     <row r="8" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>7</v>
+        <v>124</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>90</v>
+        <v>127</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>91</v>
+        <v>128</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>93</v>
+        <v>131</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>7</v>
+        <v>132</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>95</v>
+        <v>134</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>7</v>
+        <v>135</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>96</v>
+        <v>136</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>97</v>
+        <v>137</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>7</v>
+        <v>138</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>8</v>
@@ -3753,13 +3948,13 @@
     </row>
     <row r="14" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>98</v>
+        <v>139</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>7</v>
+        <v>141</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>8</v>
@@ -3767,111 +3962,111 @@
     </row>
     <row r="15" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>100</v>
+        <v>142</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>101</v>
+        <v>143</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>7</v>
+        <v>144</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>102</v>
+        <v>145</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>103</v>
+        <v>146</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>7</v>
+        <v>147</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>104</v>
+        <v>148</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>105</v>
+        <v>149</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>7</v>
+        <v>150</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>106</v>
+        <v>151</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>107</v>
+        <v>152</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>7</v>
+        <v>153</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>108</v>
+        <v>154</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>109</v>
+        <v>155</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>7</v>
+        <v>156</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>110</v>
+        <v>157</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>111</v>
+        <v>158</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>7</v>
+        <v>159</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>113</v>
+        <v>161</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>7</v>
+        <v>162</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>115</v>
+        <v>164</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>8</v>
@@ -3879,30 +4074,30 @@
     </row>
     <row r="23" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>116</v>
+        <v>165</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>117</v>
+        <v>166</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>7</v>
+        <v>167</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" ht="80" customHeight="1" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>118</v>
+        <v>168</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>119</v>
+        <v>169</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>